<commit_message>
Document branch conventions in review guidelines
</commit_message>
<xml_diff>
--- a/AI-Driven-Gated-Community-Tracker.xlsx
+++ b/AI-Driven-Gated-Community-Tracker.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rbb57ed12385d497b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="Rdfe9742e8c874ed8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="R500212ecbb4d429d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="Ree4455f286614b9a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="Rf23c7a74e81044b7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R011869dbe70b4c9a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rd8f8bdc6ba1c4232"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="R239860711d9b4b79"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="Rd9c4c0324d204813"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="R240cff2416ea43e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="R28e059673da04588"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R2dbef616c54f42da"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1027,7 +1027,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:person displayName="Akhil" id="{0ECEE2D0-4CFC-4315-AE53-3B26A1A68D6E}"/>
+  <xltc:person displayName="Akhil" id="{02555172-73D1-4429-A3EB-4954B550ECC3}"/>
 </xltc:personList>
 </file>
 
@@ -1072,7 +1072,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="ReviewGuidelines" displayName="ReviewGuidelines" ref="A5:G30" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="ReviewGuidelines" displayName="ReviewGuidelines" ref="A5:G34" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="Guideline ID"/>
     <x:tableColumn id="2" name="Area"/>
@@ -2994,7 +2994,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R092039fa58c34ec4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R71aa9ec2819f46aa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4116,7 +4116,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbec41092f5994f3f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R42fa18b8f72740a3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4750,25 +4750,117 @@
       </x:c>
     </x:row>
     <x:row r="30" ht="48" customHeight="1">
-      <x:c r="A30" s="160" t="str">
+      <x:c r="A30" s="158" t="str">
         <x:v>CR025</x:v>
       </x:c>
-      <x:c r="B30" s="160" t="str">
+      <x:c r="B30" s="158" t="str">
         <x:v>Documentation</x:v>
       </x:c>
-      <x:c r="C30" s="160" t="str">
+      <x:c r="C30" s="158" t="str">
         <x:v>Decision records</x:v>
       </x:c>
-      <x:c r="D30" s="160" t="str">
+      <x:c r="D30" s="158" t="str">
         <x:v>Document architecture, data flows, important trade-offs, operating procedures, and known limitations.</x:v>
       </x:c>
-      <x:c r="E30" s="160" t="str">
+      <x:c r="E30" s="158" t="str">
         <x:v>Reviewed ADR or repository documentation.</x:v>
       </x:c>
-      <x:c r="F30" s="160" t="str">
+      <x:c r="F30" s="158" t="str">
         <x:v>As decisions occur</x:v>
       </x:c>
-      <x:c r="G30" s="161" t="str">
+      <x:c r="G30" s="159" t="str">
+        <x:v>AKHIL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="48" customHeight="1">
+      <x:c r="A31" s="158" t="str">
+        <x:v>CR026</x:v>
+      </x:c>
+      <x:c r="B31" s="158" t="str">
+        <x:v>Version control</x:v>
+      </x:c>
+      <x:c r="C31" s="158" t="str">
+        <x:v>Feature branches</x:v>
+      </x:c>
+      <x:c r="D31" s="158" t="str">
+        <x:v>Use `feature/&lt;task-name&gt;` for planned features and tracker tasks. The task name must be concise, lowercase, and kebab-case.</x:v>
+      </x:c>
+      <x:c r="E31" s="158" t="str">
+        <x:v>Active branch name matches the task and required prefix.</x:v>
+      </x:c>
+      <x:c r="F31" s="158" t="str">
+        <x:v>Every feature task</x:v>
+      </x:c>
+      <x:c r="G31" s="159" t="str">
+        <x:v>AKHIL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="48" customHeight="1">
+      <x:c r="A32" s="158" t="str">
+        <x:v>CR027</x:v>
+      </x:c>
+      <x:c r="B32" s="158" t="str">
+        <x:v>Version control</x:v>
+      </x:c>
+      <x:c r="C32" s="158" t="str">
+        <x:v>Bug-fix branches</x:v>
+      </x:c>
+      <x:c r="D32" s="158" t="str">
+        <x:v>Use `bugfix/&lt;bugfix-name&gt;` for normal defect corrections. The defect name must be concise, lowercase, and kebab-case.</x:v>
+      </x:c>
+      <x:c r="E32" s="158" t="str">
+        <x:v>Active branch name identifies the corrected defect and required prefix.</x:v>
+      </x:c>
+      <x:c r="F32" s="158" t="str">
+        <x:v>Every bug fix</x:v>
+      </x:c>
+      <x:c r="G32" s="159" t="str">
+        <x:v>AKHIL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="48" customHeight="1">
+      <x:c r="A33" s="158" t="str">
+        <x:v>CR028</x:v>
+      </x:c>
+      <x:c r="B33" s="158" t="str">
+        <x:v>Version control</x:v>
+      </x:c>
+      <x:c r="C33" s="158" t="str">
+        <x:v>Hotfix branches</x:v>
+      </x:c>
+      <x:c r="D33" s="158" t="str">
+        <x:v>Use `hotfix/&lt;hotfix-name&gt;` only for urgent production corrections. Document urgency, impact, validation, and rollback steps.</x:v>
+      </x:c>
+      <x:c r="E33" s="158" t="str">
+        <x:v>Active branch name, incident evidence, tests, and rollback notes.</x:v>
+      </x:c>
+      <x:c r="F33" s="158" t="str">
+        <x:v>Every hotfix</x:v>
+      </x:c>
+      <x:c r="G33" s="159" t="str">
+        <x:v>AKHIL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="48" customHeight="1">
+      <x:c r="A34" s="160" t="str">
+        <x:v>CR029</x:v>
+      </x:c>
+      <x:c r="B34" s="160" t="str">
+        <x:v>Version control</x:v>
+      </x:c>
+      <x:c r="C34" s="160" t="str">
+        <x:v>Stable main branch</x:v>
+      </x:c>
+      <x:c r="D34" s="160" t="str">
+        <x:v>Keep `main` as the stable baseline. Complete work on a dedicated branch and merge only after applicable acceptance and review checks pass.</x:v>
+      </x:c>
+      <x:c r="E34" s="160" t="str">
+        <x:v>Clean review diff, passing checks, and approved merge evidence.</x:v>
+      </x:c>
+      <x:c r="F34" s="160" t="str">
+        <x:v>Every merge</x:v>
+      </x:c>
+      <x:c r="G34" s="161" t="str">
         <x:v>AKHIL</x:v>
       </x:c>
     </x:row>
@@ -4779,7 +4871,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c58e648735a445b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R101c721e24394c9b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5756,7 +5848,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R039a299b006a4ea1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb6d2d6ecca547df"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Define sitemap and user journeys
</commit_message>
<xml_diff>
--- a/AI-Driven-Gated-Community-Tracker.xlsx
+++ b/AI-Driven-Gated-Community-Tracker.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rc705db99dc6f4b48"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="R06b170952b9e443a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="R895333e5c84f499d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="R836808868b024858"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="R44f7bdbfd58b409a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R4a2e7b46a3b04973"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rebcc04a68a1946ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="Ra8013de723974ce2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="Raf1f8d2ee5394497"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="Rd26c037595b041ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="Rb8ace8e17976429c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R15c4fe74c2d84661"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1039,7 +1039,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:person displayName="Akhil" id="{51704472-2603-4CA0-9062-DCC28AB93573}"/>
+  <xltc:person displayName="Akhil" id="{FA41126D-527F-44E8-9BB1-0FE7CE6EA559}"/>
 </xltc:personList>
 </file>
 
@@ -1457,7 +1457,7 @@
       </x:c>
       <x:c r="B8" s="131" t="n">
         <x:f>COUNTIF('Phase 1 MVP'!I6:I33,"Completed")+COUNTIF('Phase 2 MVP'!I6:I30,"Completed")</x:f>
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="C8" s="120"/>
       <x:c r="D8" s="132" t="str">
@@ -1488,7 +1488,7 @@
       </x:c>
       <x:c r="B9" s="131" t="n">
         <x:f>COUNTIF('Phase 1 MVP'!I6:I33,"Planned")+COUNTIF('Phase 2 MVP'!I6:I30,"Planned")</x:f>
-        <x:v>24</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="C9" s="120"/>
       <x:c r="D9" s="120"/>
@@ -1522,7 +1522,7 @@
       </x:c>
       <x:c r="B11" s="131" t="n">
         <x:f>COUNTIF('Phase 1 MVP'!I6:I33,"In Progress")+COUNTIF('Phase 2 MVP'!I6:I30,"In Progress")</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C11" s="120"/>
       <x:c r="D11" s="120"/>
@@ -2225,16 +2225,16 @@
         <x:v>46273</x:v>
       </x:c>
       <x:c r="I10" s="150" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="J10" s="151" t="str">
         <x:v>T0003 and initial T0004 inputs</x:v>
       </x:c>
       <x:c r="K10" s="151" t="str">
-        <x:v>Confirm whether pricing and availability will be public.</x:v>
+        <x:v>Completed using the approved product brief, temporary content register, responsive scope, and future concierge requirements.</x:v>
       </x:c>
       <x:c r="L10" s="151" t="str">
-        <x:v>Planned: approve navigation and conversion journeys.</x:v>
+        <x:v>Completed: primary and footer navigation, 18 routes, homepage sequence, eight user journeys, responsive patterns, analytics events, and content ownership documented.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="54" customHeight="1">
@@ -2264,7 +2264,7 @@
         <x:v>46276</x:v>
       </x:c>
       <x:c r="I11" s="150" t="str">
-        <x:v>Planned</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="J11" s="151" t="str">
         <x:v>T0004 and T0005</x:v>
@@ -2273,7 +2273,7 @@
         <x:v>Select preferred mood, imagery style, and animation intensity.</x:v>
       </x:c>
       <x:c r="L11" s="151" t="str">
-        <x:v>Planned: approve one visual concept before detailed UI work.</x:v>
+        <x:v>In progress: translate the approved information architecture and nature-led positioning into an original visual concept for review.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="54" customHeight="1">
@@ -3158,7 +3158,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2797fd042b75430e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb9b3c4fa39f44801"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4280,7 +4280,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd05e7ce011df45cf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3966d25e75c04a7b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5035,7 +5035,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re0c3d210bc24461b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9c3b647964664c5b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6012,7 +6012,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad4e298b169846fc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5e3281d76ddf49dc"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Create tropical visual direction
</commit_message>
<xml_diff>
--- a/AI-Driven-Gated-Community-Tracker.xlsx
+++ b/AI-Driven-Gated-Community-Tracker.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rebcc04a68a1946ae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="Ra8013de723974ce2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="Raf1f8d2ee5394497"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="Rd26c037595b041ea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="Rb8ace8e17976429c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R15c4fe74c2d84661"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rd4b73ace02ee494e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="R2853f1f2b3bf4834"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="R6b561fc3baec441e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="R821ec122c689450b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="Ra4b5598a9ba14402"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="Rac032536be7c433f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1039,7 +1039,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:person displayName="Akhil" id="{FA41126D-527F-44E8-9BB1-0FE7CE6EA559}"/>
+  <xltc:person displayName="Akhil" id="{ADB9FC84-699D-4142-A2B6-BCF18A90F195}"/>
 </xltc:personList>
 </file>
 
@@ -1457,7 +1457,7 @@
       </x:c>
       <x:c r="B8" s="131" t="n">
         <x:f>COUNTIF('Phase 1 MVP'!I6:I33,"Completed")+COUNTIF('Phase 2 MVP'!I6:I30,"Completed")</x:f>
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C8" s="120"/>
       <x:c r="D8" s="132" t="str">
@@ -1488,7 +1488,7 @@
       </x:c>
       <x:c r="B9" s="131" t="n">
         <x:f>COUNTIF('Phase 1 MVP'!I6:I33,"Planned")+COUNTIF('Phase 2 MVP'!I6:I30,"Planned")</x:f>
-        <x:v>22</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="C9" s="120"/>
       <x:c r="D9" s="120"/>
@@ -2264,16 +2264,16 @@
         <x:v>46276</x:v>
       </x:c>
       <x:c r="I11" s="150" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="J11" s="151" t="str">
         <x:v>T0004 and T0005</x:v>
       </x:c>
       <x:c r="K11" s="151" t="str">
-        <x:v>Select preferred mood, imagery style, and animation intensity.</x:v>
+        <x:v>Completed using the approved product brief, sitemap, temporary reference imagery, and an original generated concept board.</x:v>
       </x:c>
       <x:c r="L11" s="151" t="str">
-        <x:v>In progress: translate the approved information architecture and nature-led positioning into an original visual concept for review.</x:v>
+        <x:v>Completed: Quiet Tropical Modernism direction defines palette, typography, layout, imagery, motifs, components, motion, responsive behavior, and prototype disclosure.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="54" customHeight="1">
@@ -2303,7 +2303,7 @@
         <x:v>46283</x:v>
       </x:c>
       <x:c r="I12" s="150" t="str">
-        <x:v>Planned</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="J12" s="151" t="str">
         <x:v>T0006 approved</x:v>
@@ -2312,7 +2312,7 @@
         <x:v>Confirm accessibility target and final brand fonts.</x:v>
       </x:c>
       <x:c r="L12" s="151" t="str">
-        <x:v>Planned: deliver reusable tokens and component specifications.</x:v>
+        <x:v>In progress: convert the approved visual direction into reusable tokens, component specifications, interaction states, responsive grids, and accessibility rules.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="54" customHeight="1">
@@ -3158,7 +3158,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb9b3c4fa39f44801"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6e7d5e754ceb4624"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4280,7 +4280,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3966d25e75c04a7b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rade809bd1d5d438d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5035,7 +5035,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9c3b647964664c5b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf4cf1aa0b3b047b9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6012,7 +6012,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5e3281d76ddf49dc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rce69cdd381f64743"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Build implementation-ready design system
</commit_message>
<xml_diff>
--- a/AI-Driven-Gated-Community-Tracker.xlsx
+++ b/AI-Driven-Gated-Community-Tracker.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rd4b73ace02ee494e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="R2853f1f2b3bf4834"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="R6b561fc3baec441e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="R821ec122c689450b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="Ra4b5598a9ba14402"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="Rac032536be7c433f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rf1d42a66d66340e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="Rd9d6236e94134c71"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="R49b41ff48296475b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="R3e4342d75c0b4ff6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="Re4f225e477074bab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="Rbe7fad4f1a984016"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1039,7 +1039,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:person displayName="Akhil" id="{ADB9FC84-699D-4142-A2B6-BCF18A90F195}"/>
+  <xltc:person displayName="Akhil" id="{89EFB53E-77CA-4E7D-9670-0C1C58658039}"/>
 </xltc:personList>
 </file>
 
@@ -1457,7 +1457,7 @@
       </x:c>
       <x:c r="B8" s="131" t="n">
         <x:f>COUNTIF('Phase 1 MVP'!I6:I33,"Completed")+COUNTIF('Phase 2 MVP'!I6:I30,"Completed")</x:f>
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C8" s="120"/>
       <x:c r="D8" s="132" t="str">
@@ -1488,7 +1488,7 @@
       </x:c>
       <x:c r="B9" s="131" t="n">
         <x:f>COUNTIF('Phase 1 MVP'!I6:I33,"Planned")+COUNTIF('Phase 2 MVP'!I6:I30,"Planned")</x:f>
-        <x:v>21</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C9" s="120"/>
       <x:c r="D9" s="120"/>
@@ -2303,16 +2303,16 @@
         <x:v>46283</x:v>
       </x:c>
       <x:c r="I12" s="150" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="J12" s="151" t="str">
         <x:v>T0006 approved</x:v>
       </x:c>
       <x:c r="K12" s="151" t="str">
-        <x:v>Confirm accessibility target and final brand fonts.</x:v>
+        <x:v>Completed using the Quiet Tropical Modernism direction, WCAG 2.2 AA target, responsive sitemap, and concierge-preview requirements.</x:v>
       </x:c>
       <x:c r="L12" s="151" t="str">
-        <x:v>In progress: convert the approved visual direction into reusable tokens, component specifications, interaction states, responsive grids, and accessibility rules.</x:v>
+        <x:v>Completed: machine-readable foundations, responsive grid, typography hierarchy, component contracts, state matrix, accessibility rules, and engineering usage policy delivered.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="54" customHeight="1">
@@ -2342,7 +2342,7 @@
         <x:v>46282</x:v>
       </x:c>
       <x:c r="I13" s="150" t="str">
-        <x:v>Planned</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="J13" s="151" t="str">
         <x:v>T0004 and T0005</x:v>
@@ -2351,7 +2351,7 @@
         <x:v>Choose CMS ownership and content approval workflow.</x:v>
       </x:c>
       <x:c r="L13" s="151" t="str">
-        <x:v>Planned: make the content model reusable by the future AI layer.</x:v>
+        <x:v>In progress: define structured, evidence-aware records for villas, amenities, plans, locations, contacts, media, documents, and references.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="54" customHeight="1">
@@ -3158,7 +3158,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6e7d5e754ceb4624"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3399813d43164bb8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4280,7 +4280,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rade809bd1d5d438d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2e1d433ce2d84bb4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5035,7 +5035,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf4cf1aa0b3b047b9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd7cd557a843b47e8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6012,7 +6012,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rce69cdd381f64743"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdcf4644420914c9c"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>